<commit_message>
docs(ai): capture des exigences DevOS — assistant vocal proactif et rappels intelligents
- REQUIREMENTS.md : FR-001→010, AC-001→012, préférences initiales, ordre de réalisation
- Analyse d'écart plateforme documentée (sandbox web vs cible Flutter/Android/Linux) : équivalents proposés, écarts assumés, aucune simulation trompeuse
- PROJECT_CONTEXT.md : produit = DevOS
- TASKS.xlsx/TASKS.md : TASK-005 terminée, TASK-006 créée et verrouillée attend signal GO
- TEAM_STATUS + DAILY_STANDUP mis à jour

Refs: TASK-005, TASK-006
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -107,8 +107,44 @@
       <color rgb="001B7D46"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <b val="1"/>
+      <color rgb="001B7D46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <color rgb="0037352F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <b val="1"/>
+      <color rgb="008C8A84"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <b val="1"/>
+      <color rgb="00D4820A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK SC"/>
+      <color rgb="001B2A4A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="008C8A84"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -157,8 +193,18 @@
         <bgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -184,6 +230,11 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="medium">
+        <color rgb="00E9E9E8"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -195,7 +246,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -305,6 +356,27 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="18" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:T12"/>
+  <dimension ref="B2:T13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -1095,13 +1167,13 @@
           <t>QA (Agent 2) + Tech Lead</t>
         </is>
       </c>
-      <c r="H9" s="31" t="inlineStr">
-        <is>
-          <t>À FAIRE</t>
+      <c r="H9" s="37" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I9" s="25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -1125,7 +1197,7 @@
       </c>
       <c r="N9" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O9" s="23" t="n">
@@ -1148,54 +1220,154 @@
       </c>
       <c r="S9" s="23" t="inlineStr">
         <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="T9" s="23" t="inlineStr">
+        <is>
+          <t>Contexte DevOS reçu ; exigences FR-001→010 + AC-001→012 + analyse d'écart plateforme enregistrées dans REQUIREMENTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="19">
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>TASK-006</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>PRODUIT</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>DevOS — Assistant vocal proactif et rappels intelligents</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>Lifecycle complet FEATURE-001 (Phase 0 UX → Phase 7 rétro)</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>Implémentation du module adapté au sandbox web (ReminderScheduler, VoiceAssistantService, NotificationService, TextToSpeechProvider, VoicePreferencesRepository, EventListener, SyncIntegration simulée, AIOrchestrator + fallback préparé) — cf. REQUIREMENTS.md §3 et §5</t>
+        </is>
+      </c>
+      <c r="G10" s="38" t="inlineStr">
+        <is>
+          <t>Équipe complète (Lead + Back + Front + QA + agents qualité)</t>
+        </is>
+      </c>
+      <c r="H10" s="39" t="inlineStr">
+        <is>
+          <t>À FAIRE</t>
+        </is>
+      </c>
+      <c r="I10" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="41" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K10" s="38" t="inlineStr">
+        <is>
+          <t>TASK-005</t>
+        </is>
+      </c>
+      <c r="L10" s="38" t="inlineStr">
+        <is>
+          <t>src/** (à créer) ; prisma/schema.prisma ; .ai/SPECS/FEATURE-001*</t>
+        </is>
+      </c>
+      <c r="M10" s="38" t="inlineStr">
+        <is>
+          <t>Gherkin AC-001→012 + E2E navigateur</t>
+        </is>
+      </c>
+      <c r="N10" s="38" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="T9" s="23" t="inlineStr">
-        <is>
-          <t>Le CTO (utilisateur) définit le produit cible ; le système exécute le lifecycle complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="25.5" customHeight="1" s="19">
-      <c r="B10" s="32" t="inlineStr">
+      <c r="O10" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q10" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R10" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S10" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T10" s="38" t="inlineStr">
+        <is>
+          <t>DÉCLENCHEMENT UNIQUEMENT À LA RÉCEPTION DU SIGNAL « GO » DU CTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1" s="19">
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
-        <is>
-          <t>5 tâches</t>
-        </is>
-      </c>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="32" t="n"/>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="32" t="n"/>
-      <c r="H10" s="32" t="n"/>
-      <c r="I10" s="33" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J10" s="32" t="n"/>
-      <c r="K10" s="32" t="n"/>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="32" t="n"/>
-      <c r="N10" s="32" t="n"/>
-      <c r="O10" s="32" t="n">
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>6 tâches</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="n"/>
+      <c r="E11" s="43" t="n"/>
+      <c r="F11" s="43" t="n"/>
+      <c r="G11" s="43" t="n"/>
+      <c r="H11" s="43" t="n"/>
+      <c r="I11" s="44" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="J11" s="43" t="n"/>
+      <c r="K11" s="43" t="n"/>
+      <c r="L11" s="43" t="n"/>
+      <c r="M11" s="43" t="n"/>
+      <c r="N11" s="43" t="n"/>
+      <c r="O11" s="43" t="n">
         <v>0</v>
       </c>
-      <c r="P10" s="32" t="n"/>
-      <c r="Q10" s="32" t="n"/>
-      <c r="R10" s="32" t="n"/>
-      <c r="S10" s="32" t="n"/>
-      <c r="T10" s="32" t="inlineStr">
-        <is>
-          <t>Terminées : 4 · En cours : 0 · À faire : 1 · Bloquées : 0</t>
+      <c r="P11" s="43" t="n"/>
+      <c r="Q11" s="43" t="n"/>
+      <c r="R11" s="43" t="n"/>
+      <c r="S11" s="43" t="n"/>
+      <c r="T11" s="43" t="inlineStr">
+        <is>
+          <t>Terminées : 5 · En cours : 0 · À faire : 1 · Bloquées : 0</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
       <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="45" t="inlineStr">
         <is>
           <t>Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
         </is>
@@ -1269,7 +1441,7 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
@@ -1284,7 +1456,7 @@
         </is>
       </c>
       <c r="C6" s="27">
-        <f>COUNTIF(TASKS!H5:H9,"TERMINÉ")</f>
+        <f>COUNTIF(TASKS!H5:H10,"TERMINÉ")</f>
         <v/>
       </c>
       <c r="D6" s="27" t="inlineStr">
@@ -1300,7 +1472,7 @@
         </is>
       </c>
       <c r="C7" s="23">
-        <f>COUNTIF(TASKS!H5:H9,"EN COURS")</f>
+        <f>COUNTIF(TASKS!H5:H10,"EN COURS")</f>
         <v/>
       </c>
       <c r="D7" s="23" t="inlineStr">
@@ -1316,7 +1488,7 @@
         </is>
       </c>
       <c r="C8" s="27">
-        <f>COUNTIF(TASKS!H5:H9,"À FAIRE")</f>
+        <f>COUNTIF(TASKS!H5:H10,"À FAIRE")</f>
         <v/>
       </c>
       <c r="D8" s="27" t="inlineStr">
@@ -1332,7 +1504,7 @@
         </is>
       </c>
       <c r="C9" s="23">
-        <f>COUNTIF(TASKS!H5:H9,"BLOQUÉ")</f>
+        <f>COUNTIF(TASKS!H5:H10,"BLOQUÉ")</f>
         <v/>
       </c>
       <c r="D9" s="23" t="inlineStr">
@@ -1348,7 +1520,7 @@
         </is>
       </c>
       <c r="C10" s="27">
-        <f>SUM(TASKS!N5:N9)</f>
+        <f>SUM(TASKS!O5:O10)</f>
         <v/>
       </c>
       <c r="D10" s="27" t="inlineStr">
@@ -1364,7 +1536,7 @@
         </is>
       </c>
       <c r="C11" s="34">
-        <f>AVERAGE(TASKS!I5:I9)</f>
+        <f>AVERAGE(TASKS!I5:I10)</f>
         <v/>
       </c>
       <c r="D11" s="23" t="inlineStr">

</xml_diff>

<commit_message>
docs(governance): durcissement sécurité soldé — DEBT-013/021 TRAITÉ, REV-004 APPROUVÉE, TASKS 17/17
- REVIEW_LOG.md : REV-004 ✅ APPROUVÉE (Agent Reviewer indépendant — FEATURE-AUTH + fix seed + durcissement ; 0 bloquant, 0 majeur, 4 mineurs tracés)
- DEBT_REPORT.md : 013 (CSP db13a8b) et 021 (rate limiting 88f334f) → TRAITÉ avec résiduels documentés ; correction arithmétique explicite des stats (17 TRAITÉ · 2 EN COURS · 1 REPORTÉ · 1 ACCEPTÉE · 1 OUVERT)
- AUDIT_REPORT.md : état des conditions du verdict AUDIT-003 (toutes soldées sauf DEBT-020 purge + verrou XFF) + focus AUDIT-004
- TASKS.xlsx (fait foi) : TASK-017, TOTAL 17/17 100 %, STATISTIQUES 5:21 — pipeline recalc/audit/scan/validate 100 % vert ; TASKS.md miroir synchronisé
- CHANGELOG : 0.5.0-security-hardening
- COMMIT_LOG : 88f334f + db13a8b consignés
- worklog.md : sections Task 26+28 (preuves throttle/CSP) — remarque du reviewer REV-004 traitée
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="202">
   <si>
     <t xml:space="preserve">Backlog Central — Système Multi-Agents</t>
   </si>
@@ -527,13 +527,46 @@
     <t xml:space="preserve">0 CRITIQUE · 2 MAJEUR · 5 MINEUR · dette 22 items (14 TRAITÉ) · restant avant prod réelle : CSP (DEBT-013) + rate limiting (DEBT-021) + purge 6 comptes de démo (DEBT-020)</t>
   </si>
   <si>
+    <t xml:space="preserve">TASK-017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DevOS — Authentification (FEATURE-AUTH, Task 26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durcissement sécurité pré-prod : rate limiting (DEBT-021) + CSP (DEBT-013) + REV-004 (Task 27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suite du plan d'action AUDIT-003 : src/lib/rate-limit.ts (fenêtre fixe mémoire, login 10/15 min/IP, register 5/h/IP, 429 uniforme { error } + Retry-After, 0 middleware/0 dépendance) ; CSP 9 directives dans next.config.ts (unsafe-inline/eval justifiés, frame-ancestors 'none', XFO SAMEORIGIN→DENY) ; revue indépendante REV-004 (Agent Reviewer) sur FEATURE-AUTH + fix seed + durcissement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORCHESTRATEUR (CTO) + AGENT REVIEWER (indépendant)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan d'action AUDIT-003 (actions 1, 2, 4, 5), DEBT-013, DEBT-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/lib/rate-limit.ts; src/lib/api-helpers.ts; src/app/api/auth/{login,register}/route.ts; next.config.ts; .ai/REVIEW_LOG.md (REV-004)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saturation curl : login 10 autorisées (1 succès navigateur + 9×401) puis 429 Retry-After 877 s, register 5×400 puis 429, métier non affecté (tasks 401, health 200) · CSP : navigation complète AuthGate→connexion→3 onglets→déconnexion 0 violation console, HMR opérationnel · lint 0 · tsc 0 · REV-004 : 2 appels auth sous throttle (429 + Retry-After 643 = comportement correct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">88f334f (rate limiting), db13a8b (CSP) — REV-004 : 0 code modifié (audit pur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REV-004 ✅ APPROUVÉE — 0 bloquant · 0 majeur · 4 mineurs tracés (XFF accès direct, Map &gt; 5000, mdp démo, h1 AuthGate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dette 22 items : 17 TRAITÉ (013/021 soldés) · 2 EN COURS (003, 017) · 1 REPORTÉ (010) · 1 ACCEPTÉE (012) · 1 OUVERT (018) · restant avant exposition prod réelle : DEBT-020 purge comptes de démo + verrou accès direct :3000 (mineur REV-004)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">16 tâches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminées : 16 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
+    <t xml:space="preserve">17 tâches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminées : 17 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
   </si>
   <si>
     <t xml:space="preserve">Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
@@ -587,7 +620,7 @@
     <t xml:space="preserve">Score santé projet</t>
   </si>
   <si>
-    <t xml:space="preserve">77 / 100 (AUDIT-003) · AUTORISÉ SOUS CONDITION (conditions 022/019 soldées)</t>
+    <t xml:space="preserve">77 / 100 (AUDIT-003) · AUTORISÉ SOUS CONDITION — toutes conditions soldées + REV-004 APPROUVÉE</t>
   </si>
   <si>
     <t xml:space="preserve">.ai/AUDIT_REPORT.md</t>
@@ -596,7 +629,7 @@
     <t xml:space="preserve">Dette technique (items)</t>
   </si>
   <si>
-    <t xml:space="preserve">.ai/DEBT_REPORT.md (14 TRAITÉ · 3 EN COURS · 1 REPORTÉ · 1 ACCEPTÉE · 3 OUVERTS)</t>
+    <t xml:space="preserve">.ai/DEBT_REPORT.md (17 TRAITÉ · 2 EN COURS · 1 REPORTÉ · 1 ACCEPTÉE · 1 OUVERT)</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1199,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:T23"/>
+  <dimension ref="B2:T24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -2160,7 +2193,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
         <v>156</v>
       </c>
@@ -2220,39 +2253,98 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="23" t="n">
+      <c r="E21" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="22" t="n">
+      <c r="J21" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O21" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="P21" s="22"/>
-      <c r="Q21" s="22"/>
-      <c r="R21" s="22"/>
-      <c r="S21" s="22"/>
-      <c r="T21" s="22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="24" t="s">
-        <v>170</v>
+      <c r="P21" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q21" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="R21" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="S21" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="22"/>
+      <c r="Q22" s="22"/>
+      <c r="R22" s="22"/>
+      <c r="S22" s="22"/>
+      <c r="T22" s="22" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="24" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2295,7 +2387,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2303,118 +2395,118 @@
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="C6" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H20,"TERMINÉ")</f>
-        <v>16</v>
+        <f aca="false">COUNTIF(TASKS!H5:H21,"TERMINÉ")</f>
+        <v>17</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H20,"EN COURS")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H21,"EN COURS")</f>
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="C8" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H20,"À FAIRE")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H21,"À FAIRE")</f>
         <v>0</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H20,"BLOQUÉ")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H21,"BLOQUÉ")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C10" s="9" t="n">
-        <f aca="false">SUM(TASKS!O5:O20)</f>
+        <f aca="false">SUM(TASKS!O5:O21)</f>
         <v>0</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="C11" s="25" t="n">
-        <f aca="false">AVERAGE(TASKS!I5:I20)</f>
+        <f aca="false">AVERAGE(TASKS!I5:I21)</f>
         <v>1</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="C13" s="27" t="n">
         <v>22</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ui) responsivité mobile vue de connexion (AuthGate) — TASK-018
- min-h-dvh + centrage sûr (my-auto remplace justify-center) : hauteur
  réduite (clavier iOS, paysage) → haut du formulaire atteignable
- paddings scoped 320 px (px-4 sm:px-6 header/content, gap/py 4 sm:6)
- h1 sr-only (partie h1 DEBT-017) ; écran chargement min-h-dvh
- preuves : hasHScroll=false 320→1280, paysage 667×375 cardTop=40 au
  scroll-top, E2E mobile connexion démo, 8 captures before/after
- env : JWT_SECRET régénéré + seed rejoué (dérive auto-sauvegarde)
- gouvernance : TASKS 18/18 (xlsx validate passed), DEBT-017 h1 soldé
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="214">
   <si>
     <t xml:space="preserve">Backlog Central — Système Multi-Agents</t>
   </si>
@@ -560,13 +560,49 @@
     <t xml:space="preserve">Dette 22 items : 17 TRAITÉ (013/021 soldés) · 2 EN COURS (003, 017) · 1 REPORTÉ (010) · 1 ACCEPTÉE (012) · 1 OUVERT (018) · restant avant exposition prod réelle : DEBT-020 purge comptes de démo + verrou accès direct :3000 (mineur REV-004)</t>
   </si>
   <si>
+    <t xml:space="preserve">TASK-018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsivité mobile de la vue de connexion (AuthGate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exigence CTO « assure-toi de la responsivité mobile de la vue de connexion ». Analyse statique (auth-gate.tsx, input/card/tabs/toast, layout) + tests navigateur multi-viewports (375 / 320 / 667×375 paysage / 1280). Correctifs : (1) min-h-dvh + centrage « sûr » my-auto (remplace justify-center : en hauteur réduite — clavier iOS, paysage — le haut du formulaire reste atteignable au scroll, plus de contenu clippé) ; (2) paddings scoped px-4 sm:px-6 sur CardHeader/CardContent + gap-4/py-4 sm:gap-6/sm:py-6 (rythme 320 px) ; (3) h1 sr-only (partie h1 de DEBT-017) ; écran de chargement aligné en min-h-dvh. Aucun changement de comportement fonctionnel ni de contrat API.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend / UX (CTO Task 29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TASK-015 (FEATURE-AUTH — la vue de connexion existe)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/components/assistant/auth-gate.tsx; tool-results/task29-mobile-375-before.png; tool-results/task29-mobile-320-before.png; tool-results/task29-mobile-375-after.png; tool-results/task29-mobile-320-after.png; tool-results/task29-mobile-landscape-after.png; tool-results/task29-desktop-after.png; tool-results/task29-mobile-login-ok.png; worklog.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hasHScroll=false à 320/375/667/1280 · paysage 667×375 : docH 606 &gt; viewport 375, scroll-top → cardTop=40 px (haut du formulaire visible — centrage sûr prouvé) · computed minHeight=100dvh · h1 sr-only présent (position absolute) · E2E mobile complet : connexion demo@devos.test → « Bienvenue, Démonstration DevOS ! » + app shell (Assistant/Tâches/Paramètres) · 0 erreur console · toast mobile top full-width observé live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 middleware respecté (ADR-003) · aucun composant ui/ global modifié (overrides scoped à l'instance AuthForm) · dérive environnement détectée et corrigée en passant : .env sans JWT_SECRET (restauration env) → secret régénéré + User table vide → seed rejoué (comptes auto-sauvegarde, cf. COMMIT_LOG §auto-sauvegarde)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vue de connexion : 100 % utilisable 320→1280 px, clavier iOS et paysage couverts (centrage sûr) · a11y : h1 ajouté (partie de DEBT-017 — le découpage UI reste EN COURS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min-h-dvh : dégradation gracieuse top-alignée sur navigateurs sans dvh (&lt; 2022) — acceptable · AUDIT-004 requis après cette évolution (règle « audit après chaque feature »)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">17 tâches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminées : 17 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
+    <t xml:space="preserve">18 tâches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminées : 18 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
   </si>
   <si>
     <t xml:space="preserve">Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
@@ -1199,7 +1235,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:T24"/>
+  <dimension ref="B2:T25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -2312,39 +2348,98 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="23" t="n">
+      <c r="F22" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="22" t="n">
+      <c r="J22" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="K22" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O22" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="P22" s="22"/>
-      <c r="Q22" s="22"/>
-      <c r="R22" s="22"/>
-      <c r="S22" s="22"/>
-      <c r="T22" s="22" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="24" t="s">
-        <v>181</v>
+      <c r="P22" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q22" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="R22" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="S22" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="T22" s="9" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="22"/>
+      <c r="Q23" s="22"/>
+      <c r="R23" s="22"/>
+      <c r="S23" s="22"/>
+      <c r="T23" s="22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="24" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2387,7 +2482,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2395,118 +2490,118 @@
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C6" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H21,"TERMINÉ")</f>
-        <v>17</v>
+        <f aca="false">COUNTIF(TASKS!H5:H22,"TERMINÉ")</f>
+        <v>18</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H21,"EN COURS")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H22,"EN COURS")</f>
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="C8" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H21,"À FAIRE")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H22,"À FAIRE")</f>
         <v>0</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H21,"BLOQUÉ")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H22,"BLOQUÉ")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C10" s="9" t="n">
-        <f aca="false">SUM(TASKS!O5:O21)</f>
+        <f aca="false">SUM(TASKS!O5:O22)</f>
         <v>0</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="C11" s="25" t="n">
-        <f aca="false">AVERAGE(TASKS!I5:I21)</f>
+        <f aca="false">AVERAGE(TASKS!I5:I22)</f>
         <v>1</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C13" s="27" t="n">
         <v>22</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ui-shell): vues pleine largeur (w-full) + navigation mobile tiroir seul — TASK-020
- main : mx-auto max-w-5xl → w-full (preuves 1280/1920 px, max-width none)
- BottomNav (barre compacte 5 destinations) supprimée : composant, champ
  mobilePrimary, export MOBILE_PRIMARY_ITEMS, dégagements pb-24/+4,5rem
- Navigation mobile = tiroir (Sheet) seul — amendement ADR-004 §4
- Registre navigation.ts à source unique conservé (sidebar + tiroir)
- E2E : mobile 375 bottomNavPresent=false, tiroir 11+5 destinations
  opérationnel, hasHScroll=false · lint 0 · tsc 0
- Gouvernance : TASKS 20/20 (validate passed), TASKS.md, ADR-004, worklog
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="236">
   <si>
     <t xml:space="preserve">Backlog Central — Système Multi-Agents</t>
   </si>
@@ -629,13 +629,46 @@
     <t xml:space="preserve">Périmètre volontairement MVP (recommandation CTO §6) · AUDIT-005 requis après cette feature · DEBT-017 : settings-screen.tsx (632) reste à découper</t>
   </si>
   <si>
+    <t xml:space="preserve">TASK-020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DevOS — Espace de travail (FEATURE-UI-SHELL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vues en pleine largeur (w-full) sur web + navigation mobile réduite au tiroir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exigence CTO « Mets les vues en w-full pour web, en mobile, retire le menu compacte, garde juste la sidebar (drawer) ». (1) main passe de mx-auto max-w-5xl à w-full (preuves mesurées : 1280 → main 1024 px = 1280−256 sidebar ; 1920 → main 1664 px, max-width none, marges 0) ; footer aligné w-full. (2) BottomNav (barre inférieure 5 destinations) supprimée : composant bottom-nav.tsx supprimé, champ mobilePrimary + export MOBILE_PRIMARY_ITEMS retirés du registre navigation.ts, dégagements retirés (pb-24 sur main, +4,5rem sur footer). (3) Navigation mobile = tiroir (Sheet) seul via burger header : E2E 375 px — bottomNavPresent=false, burger visible, tiroir complet (11 actives + 5 « Bientôt »), navigation Projets OK avec fermeture auto. ADR-004 amendé (§4). Aucun changement de contrat API.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend / UX (CTO Task 35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TASK-019 (FEATURE-UI-SHELL — le shell et la navigation existent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/components/shell/app-shell.tsx; src/lib/navigation.ts; src/components/shell/bottom-nav.tsx (supprimé); .ai/ADR/ADR-004-shell-navigation-permissions.md; tool-results/task20-desktop-wfull.png; tool-results/task20-desktop-1920-wfull.png; tool-results/task20-mobile-drawer.png; tool-results/task20-mobile-projets.png; worklog.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desktop 1280 : mainW=1024 (= viewport−sidebar 256), mainMaxW=none, marges 0 · Desktop 1920 : mainW=1664, footerW=1664, footerMaxW=none · Mobile 375 : bottomNavPresent=false, burger présent+visible, mainW=375, hasHScroll=false · E2E tiroir : ouverture → navigation complète visible → clic Projets → h1 « Projets » + tiroir fermé · lint 0 · tsc 0 · 0 erreur console (2 warnings Radix DialogContent préexistants, hors périmètre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 middleware respecté (ADR-003) · registre à source unique conservé (sidebar + tiroir générés depuis NAV_SECTIONS — aucune duplication) · a11y : navigation tiroir aria-labelée, aria-current conservé, cibles ≥ 44 px (min-h-11) · suppression fichier = dette code réduite (−76 l. bottom-nav.tsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web : vues exploitent toute la largeur disponible (fini la colonne max-w-5xl) · Mobile : navigation unifiée tiroir (une seule source de vérité visuelle), moins de chrome à l'écran · MOBILE_PRIMARY_ITEMS retiré — breaking change interne sans impact externe (aucun autre consommateur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUDIT-006 requis après cette évolution (règle « audit après chaque feature ») · le cahier des charges initial §5 (barre inférieure 5 destinations) est officiellement supplanté par l'amendement ADR-004 §4</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">19 tâches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminées : 19 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
+    <t xml:space="preserve">20 tâches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminées : 20 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
   </si>
   <si>
     <t xml:space="preserve">Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
@@ -1268,7 +1301,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:T26"/>
+  <dimension ref="B2:T27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -2499,39 +2532,98 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="23" t="n">
+      <c r="E24" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="22"/>
-      <c r="O24" s="22" t="n">
+      <c r="J24" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="K24" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="M24" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O24" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="22"/>
-      <c r="R24" s="22"/>
-      <c r="S24" s="22"/>
-      <c r="T24" s="22" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="24" t="s">
-        <v>204</v>
+      <c r="P24" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q24" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="R24" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="S24" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="T24" s="9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="22"/>
+      <c r="Q25" s="22"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="22" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="24" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2574,7 +2666,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2582,118 +2674,118 @@
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="C6" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H23,"TERMINÉ")</f>
-        <v>19</v>
+        <f aca="false">COUNTIF(TASKS!H5:H24,"TERMINÉ")</f>
+        <v>20</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H23,"EN COURS")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H24,"EN COURS")</f>
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C8" s="9" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H23,"À FAIRE")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H24,"À FAIRE")</f>
         <v>0</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">COUNTIF(TASKS!H5:H23,"BLOQUÉ")</f>
+        <f aca="false">COUNTIF(TASKS!H5:H24,"BLOQUÉ")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="C10" s="9" t="n">
-        <f aca="false">SUM(TASKS!O5:O23)</f>
+        <f aca="false">SUM(TASKS!O5:O24)</f>
         <v>0</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="C11" s="25" t="n">
-        <f aca="false">AVERAGE(TASKS!I5:I23)</f>
+        <f aca="false">AVERAGE(TASKS!I5:I24)</f>
         <v>1</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="C13" s="27" t="n">
         <v>22</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(governance): TASK-025 consignée (25/25) + INC-003 + leçons + COMMIT_LOG Task 40
- TASKS.xlsx: TASK-025 ligne 29, TOTAL 30 « 25 tâches », STATISTIQUES 5:29
  (intégrité: 25 IDs uniques, 25/25 TERMINÉ) + TASKS.md miroir synchronisé
- INCIDENTS.md: INC-003 — 3e occurrence du pattern INC-001 (DB + .env non
  persistants entre sessions); chantier « sauvegardes » priorisé
- LESSONS_LEARNED: +3 leçons (credential communiqué au canal, export état
  fin de session, diagnostic par diff d'attributs d'hydratation)
- COMMIT_LOG: section Task 40 (275603b) + complétion placeholder Task 38
  (f00c40d) + constat d'intégrité: TASK-024 n'avait jamais été poussée
- worklog.md: section Task 40 + constat push Task 38 inexact, corrigé
- purge: tool-results/read_*.txt (artefact de lecture hérité)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:T31"/>
+  <dimension ref="A2:T32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="28" min="1" max="1"/>
@@ -2985,45 +2985,138 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="29">
-      <c r="B29" s="50" t="inlineStr">
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>TASK-025</t>
+        </is>
+      </c>
+      <c r="C29" s="37" t="inlineStr">
+        <is>
+          <t>GOUVERNANCE</t>
+        </is>
+      </c>
+      <c r="D29" s="37" t="inlineStr">
+        <is>
+          <t>DevOS — Incident INC-003 (accès CTO + hydratation)</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="inlineStr">
+        <is>
+          <t>Restauration du compte akoun@devos.test (base SQLite perdue au re-provisionnement de session) + neutralisation du warning d'hydratation (attributs d'extension navigateur)</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>Signalement CTO « le compte de connexion ne fonctionne plus » + console hydration mismatch (bis_skin_checked / bis_register / __processed_*). Diagnostic AVANT action : (1) dev.log — POST /api/auth/login 401 avec SELECT User exécuté sans erreur → identifiants refusés ; (2) inspection DB READ-ONLY — 0 utilisateur, 0 tâche, 0 projet, 0 conversation, 0 automatisation : db/custom.db recréée VIDE (mtime 16:27 &gt; xlsx gouvernance 13:09) au re-provisionnement de la session — la base locale n'est pas versionnée (risque « sauvegardes » tracé au backlog) ; (3) hydration — les seuls attributs en diff portent les signatures d'extension navigateur (Bitdefender : bis_*) : aucun diff applicatif, cause externe confirmée. Remédiation : compte CTO recréé (bcryptjs coût 10, mot de passe transmis au CTO dans le canal privé, JAMAIS commité) ; suppressHydrationWarning ajouté sur &lt;body&gt; (couvre l'élément racine ; recommandation CTO : désactiver l'extension sur ce site ou utiliser une fenêtre privée — React ne peut pas empêcher une extension de muter le DOM avant hydratation) ; INC-003 consigné (INCIDENTS.md) + leçons (LESSONS_LEARNED) : toute réinitialisation de credential doit être communiquée immédiatement au CTO ; la DB locale doit être sauvegardée avant toute fin de session (backlog sauvegardes).</t>
+        </is>
+      </c>
+      <c r="G29" s="37" t="inlineStr">
+        <is>
+          <t>ORCHESTRATEUR (CTO Task 40)</t>
+        </is>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I29" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="39" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K29" s="37" t="inlineStr">
+        <is>
+          <t>AUDIT-007 (83,8/100) — session Task 38 : credential réinitialisé pour E2E sans transmission explicite ; base perdue entre sessions</t>
+        </is>
+      </c>
+      <c r="L29" s="37" t="inlineStr">
+        <is>
+          <t>src/app/layout.tsx; .zscripts/task25_check_users.ts; .zscripts/task25_reset_akoun.ts; .ai/INCIDENTS.md; .ai/LESSONS_LEARNED.md; .ai/TASKS.md; worklog.md; tool-results/task25-login-ok.png; tool-results/task25-intelligence-vue.png</t>
+        </is>
+      </c>
+      <c r="M29" s="37" t="inlineStr">
+        <is>
+          <t>curl : POST /api/auth/login akoun@devos.test → 200 + cookie devos_session · GET /api/auth/me → 200 (id/email corrects) · E2E agent-browser : login UI → vue « DevOS Intelligence » rendue (captures), sidebar + tiroir mobile OK, 0 erreur console bloquante · lint 0 · tsc 0 · intégrité xlsx : 25 IDs uniques 5-29, TOTAL 30 « 25 tâches », STATISTIQUES 5:29</t>
+        </is>
+      </c>
+      <c r="N29" s="37" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O29" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="37" t="inlineStr">
+        <is>
+          <t>Mot de passe CTO jamais commité (transmis par canal privé + hachage bcrypt coût 10) · aucune modification backend (0 endpoint touché — contrat v1.4 intact) · layout.tsx : attribut suppressHydrationWarning uniquement, aucun changement de comportement · diagnostic fondé sur preuves (dev.log, inspection DB, signatures d'attributs) — aucune modification aveugle</t>
+        </is>
+      </c>
+      <c r="Q29" s="37" t="inlineStr">
+        <is>
+          <t>Accès CTO restauré sans perte d'intégrité : le compte existant étant définitivement perdu avec la base, une recréation propre était la seule voie · la refonte DevOS Intelligence (TASK-024, be695aa) est confirmée présente et fonctionnelle après restauration du login</t>
+        </is>
+      </c>
+      <c r="R29" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="S29" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="T29" s="37" t="inlineStr">
+        <is>
+          <t>Les données utilisateur antérieures (conversations, automatisations) sont définitivement perdues avec l'ancienne base — recommandation : activer le chantier « sauvegardes » (backlog) avant les prochaines itérations · suppression d'extension navigateur recommandée pour éliminer tout warning résiduel sur les éléments internes (suppressHydrationWarning ne couvre que l'élément porteur)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="29">
+      <c r="B30" s="50" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C29" s="50" t="inlineStr">
-        <is>
-          <t>24 tâches</t>
-        </is>
-      </c>
-      <c r="D29" s="50" t="n"/>
-      <c r="E29" s="50" t="n"/>
-      <c r="F29" s="50" t="n"/>
-      <c r="G29" s="50" t="n"/>
-      <c r="H29" s="50" t="n"/>
-      <c r="I29" s="51" t="n">
+      <c r="C30" s="50" t="inlineStr">
+        <is>
+          <t>25 tâches</t>
+        </is>
+      </c>
+      <c r="D30" s="50" t="n"/>
+      <c r="E30" s="50" t="n"/>
+      <c r="F30" s="50" t="n"/>
+      <c r="G30" s="50" t="n"/>
+      <c r="H30" s="50" t="n"/>
+      <c r="I30" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="J29" s="50" t="n"/>
-      <c r="K29" s="50" t="n"/>
-      <c r="L29" s="50" t="n"/>
-      <c r="M29" s="50" t="n"/>
-      <c r="N29" s="50" t="n"/>
-      <c r="O29" s="50" t="n">
+      <c r="J30" s="50" t="n"/>
+      <c r="K30" s="50" t="n"/>
+      <c r="L30" s="50" t="n"/>
+      <c r="M30" s="50" t="n"/>
+      <c r="N30" s="50" t="n"/>
+      <c r="O30" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="P29" s="50" t="n"/>
-      <c r="Q29" s="50" t="n"/>
-      <c r="R29" s="50" t="n"/>
-      <c r="S29" s="50" t="n"/>
-      <c r="T29" s="50" t="inlineStr">
-        <is>
-          <t>Terminées : 24 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="29"/>
-    <row r="31" ht="15" customHeight="1" s="29">
-      <c r="B31" s="52" t="inlineStr">
+      <c r="P30" s="50" t="n"/>
+      <c r="Q30" s="50" t="n"/>
+      <c r="R30" s="50" t="n"/>
+      <c r="S30" s="50" t="n"/>
+      <c r="T30" s="50" t="inlineStr">
+        <is>
+          <t>Terminées : 25 · En cours : 0 · À faire : 0 · Bloquées : 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="29"/>
+    <row r="32" ht="15" customHeight="1" s="29">
+      <c r="B32" s="52" t="inlineStr">
         <is>
           <t>Règles de dépendance : Frontend bloqué tant que contrat API non validé · Backend bloqué sur auth/permissions tant que Security non validé · Aucune tâche TERMINÉE sans commits propres + revue positive · Frontend : + validation a11y + perf · Aucune livraison PROD sans audit global ≥ 60/100.</t>
         </is>
@@ -3096,7 +3189,7 @@
         </is>
       </c>
       <c r="C5" s="33" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
@@ -3111,7 +3204,7 @@
         </is>
       </c>
       <c r="C6" s="37">
-        <f>COUNTIF(TASKS!H5:H28,"TERMINÉ")</f>
+        <f>COUNTIF(TASKS!H5:H29,"TERMINÉ")</f>
         <v/>
       </c>
       <c r="D6" s="37" t="inlineStr">
@@ -3127,7 +3220,7 @@
         </is>
       </c>
       <c r="C7" s="33">
-        <f>COUNTIF(TASKS!H5:H28,"EN COURS")</f>
+        <f>COUNTIF(TASKS!H5:H29,"EN COURS")</f>
         <v/>
       </c>
       <c r="D7" s="33" t="inlineStr">
@@ -3143,7 +3236,7 @@
         </is>
       </c>
       <c r="C8" s="37">
-        <f>COUNTIF(TASKS!H5:H28,"À FAIRE")</f>
+        <f>COUNTIF(TASKS!H5:H29,"À FAIRE")</f>
         <v/>
       </c>
       <c r="D8" s="37" t="inlineStr">
@@ -3159,7 +3252,7 @@
         </is>
       </c>
       <c r="C9" s="33">
-        <f>COUNTIF(TASKS!H5:H28,"BLOQUÉ")</f>
+        <f>COUNTIF(TASKS!H5:H29,"BLOQUÉ")</f>
         <v/>
       </c>
       <c r="D9" s="33" t="inlineStr">
@@ -3175,7 +3268,7 @@
         </is>
       </c>
       <c r="C10" s="37">
-        <f>SUM(TASKS!O5:O28)</f>
+        <f>SUM(TASKS!O5:O29)</f>
         <v/>
       </c>
       <c r="D10" s="37" t="inlineStr">
@@ -3191,7 +3284,7 @@
         </is>
       </c>
       <c r="C11" s="53">
-        <f>AVERAGE(TASKS!I5:I28)</f>
+        <f>AVERAGE(TASKS!I5:I29)</f>
         <v/>
       </c>
       <c r="D11" s="33" t="inlineStr">

</xml_diff>